<commit_message>
mappings: three more confirmed, through to the StructureDefinitions
196 of 643 elements now carry a glossary code across 37 of 41 models. Two rows
remain proposed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/xls/BeModelAllergyIntolerance.xlsx
+++ b/models/xls/BeModelAllergyIntolerance.xlsx
@@ -504,7 +504,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -940,23 +939,11 @@
           <t>Data Element</t>
         </is>
       </c>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Common Glossary</t>
         </is>
       </c>
-      <c r="O1" s="1" t="n"/>
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Example Value</t>
@@ -1265,6 +1252,16 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>equivalent</t>
         </is>
       </c>
     </row>

</xml_diff>